<commit_message>
Price for Indian students: $5 list, ~₹180 in India via Gumroad PPP
- $5 personal / $20 batch licence (up to 30 students); PPP at Gumroad's
  60% maximum so India sees about ₹180 / ₹700 in rupees, with UPI
- Free copy on request for students who can't pay (STUDENTAID, 20 uses)
- Channel tracking via UTM links instead of discount codes (PPP and
  codes don't stack on Gumroad)
- Financial model uses Gumroad's published processing and refund rules
- Dashboard tracks India orders, batch licences and free copies
- Licence text covers the batch tier; sample PDF shows the price

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q1vimjhczAVgRxbbW9XqPG
</commit_message>
<xml_diff>
--- a/business/phd-atlas/ops/Business-Dashboard.xlsx
+++ b/business/phd-atlas/ops/Business-Dashboard.xlsx
@@ -632,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -662,19 +662,26 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>'Forecast' is the base-case model from research/financials.py. It is NOT actual data.</t>
+          <t>'Forecast' is the scenario model from research/financials.py ($5 list; about $2 in India via Gumroad PPP). It is NOT actual data.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>'Hours' is your study-permit self-employment log. Count every business hour.</t>
+          <t>Free copies sent with STUDENTAID count as neither paid orders nor revenue.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>'Hours' is your study-permit self-employment log. Count every business hour.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Never type estimates into 'Weekly actuals'. Leave a cell blank if you don't know.</t>
         </is>
@@ -691,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -702,12 +709,15 @@
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -753,12 +763,12 @@
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>Code NETWORK</t>
+          <t>Network orders (UTM whatsapp + group)</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>Code REDDIT</t>
+          <t>Reddit orders (UTM)</t>
         </is>
       </c>
       <c r="K1" s="3" t="inlineStr">
@@ -777,6 +787,21 @@
         </is>
       </c>
       <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>Orders from India</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Batch licences sold</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>Free copies sent (STUDENTAID)</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -799,6 +824,9 @@
       <c r="L2" s="5" t="n"/>
       <c r="M2" s="5" t="n"/>
       <c r="N2" s="5" t="n"/>
+      <c r="O2" s="5" t="n"/>
+      <c r="P2" s="5" t="n"/>
+      <c r="Q2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -817,6 +845,9 @@
       <c r="L3" s="5" t="n"/>
       <c r="M3" s="5" t="n"/>
       <c r="N3" s="5" t="n"/>
+      <c r="O3" s="5" t="n"/>
+      <c r="P3" s="5" t="n"/>
+      <c r="Q3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -835,6 +866,9 @@
       <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="n"/>
       <c r="N4" s="5" t="n"/>
+      <c r="O4" s="5" t="n"/>
+      <c r="P4" s="5" t="n"/>
+      <c r="Q4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -853,6 +887,9 @@
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
+      <c r="O5" s="5" t="n"/>
+      <c r="P5" s="5" t="n"/>
+      <c r="Q5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -871,6 +908,9 @@
       <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="n"/>
       <c r="N6" s="5" t="n"/>
+      <c r="O6" s="5" t="n"/>
+      <c r="P6" s="5" t="n"/>
+      <c r="Q6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -889,6 +929,9 @@
       <c r="L7" s="5" t="n"/>
       <c r="M7" s="5" t="n"/>
       <c r="N7" s="5" t="n"/>
+      <c r="O7" s="5" t="n"/>
+      <c r="P7" s="5" t="n"/>
+      <c r="Q7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -907,6 +950,9 @@
       <c r="L8" s="5" t="n"/>
       <c r="M8" s="5" t="n"/>
       <c r="N8" s="5" t="n"/>
+      <c r="O8" s="5" t="n"/>
+      <c r="P8" s="5" t="n"/>
+      <c r="Q8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -925,6 +971,9 @@
       <c r="L9" s="5" t="n"/>
       <c r="M9" s="5" t="n"/>
       <c r="N9" s="5" t="n"/>
+      <c r="O9" s="5" t="n"/>
+      <c r="P9" s="5" t="n"/>
+      <c r="Q9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -943,6 +992,9 @@
       <c r="L10" s="5" t="n"/>
       <c r="M10" s="5" t="n"/>
       <c r="N10" s="5" t="n"/>
+      <c r="O10" s="5" t="n"/>
+      <c r="P10" s="5" t="n"/>
+      <c r="Q10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -961,6 +1013,9 @@
       <c r="L11" s="5" t="n"/>
       <c r="M11" s="5" t="n"/>
       <c r="N11" s="5" t="n"/>
+      <c r="O11" s="5" t="n"/>
+      <c r="P11" s="5" t="n"/>
+      <c r="Q11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -979,6 +1034,9 @@
       <c r="L12" s="5" t="n"/>
       <c r="M12" s="5" t="n"/>
       <c r="N12" s="5" t="n"/>
+      <c r="O12" s="5" t="n"/>
+      <c r="P12" s="5" t="n"/>
+      <c r="Q12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -997,6 +1055,9 @@
       <c r="L13" s="5" t="n"/>
       <c r="M13" s="5" t="n"/>
       <c r="N13" s="5" t="n"/>
+      <c r="O13" s="5" t="n"/>
+      <c r="P13" s="5" t="n"/>
+      <c r="Q13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -1050,6 +1111,18 @@
       </c>
       <c r="M14" s="6">
         <f>SUM(M2:M13)</f>
+        <v/>
+      </c>
+      <c r="N14" s="6">
+        <f>SUM(N2:N13)</f>
+        <v/>
+      </c>
+      <c r="O14" s="6">
+        <f>SUM(O2:O13)</f>
+        <v/>
+      </c>
+      <c r="P14" s="6">
+        <f>SUM(P2:P13)</f>
         <v/>
       </c>
     </row>
@@ -1333,31 +1406,31 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>9.75</v>
+        <v>2.6</v>
       </c>
       <c r="E2" t="n">
-        <v>48.75</v>
+        <v>26</v>
       </c>
       <c r="F2" t="n">
-        <v>10.29</v>
+        <v>10.75</v>
       </c>
       <c r="G2" t="n">
-        <v>4.88</v>
+        <v>2.08</v>
       </c>
       <c r="H2" t="n">
-        <v>0.67</v>
+        <v>0.26</v>
       </c>
       <c r="I2" t="n">
-        <v>32.91</v>
+        <v>12.91</v>
       </c>
       <c r="J2" t="n">
         <v>12</v>
       </c>
       <c r="K2" t="n">
-        <v>2.74</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="3">
@@ -1372,31 +1445,31 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D3" t="n">
-        <v>9.75</v>
+        <v>2.6</v>
       </c>
       <c r="E3" t="n">
-        <v>292.5</v>
+        <v>130</v>
       </c>
       <c r="F3" t="n">
-        <v>61.73</v>
+        <v>53.73</v>
       </c>
       <c r="G3" t="n">
-        <v>29.25</v>
+        <v>10.4</v>
       </c>
       <c r="H3" t="n">
-        <v>4.03</v>
+        <v>1.32</v>
       </c>
       <c r="I3" t="n">
-        <v>197.49</v>
+        <v>64.55</v>
       </c>
       <c r="J3" t="n">
         <v>30</v>
       </c>
       <c r="K3" t="n">
-        <v>6.58</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="4">
@@ -1411,31 +1484,31 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="D4" t="n">
-        <v>10.5</v>
+        <v>2.75</v>
       </c>
       <c r="E4" t="n">
-        <v>262.5</v>
+        <v>110</v>
       </c>
       <c r="F4" t="n">
-        <v>55.86</v>
+        <v>44.06</v>
       </c>
       <c r="G4" t="n">
-        <v>18.38</v>
+        <v>5.5</v>
       </c>
       <c r="H4" t="n">
-        <v>3.77</v>
+        <v>1.21</v>
       </c>
       <c r="I4" t="n">
-        <v>184.5</v>
+        <v>59.23</v>
       </c>
       <c r="J4" t="n">
         <v>14</v>
       </c>
       <c r="K4" t="n">
-        <v>13.18</v>
+        <v>4.23</v>
       </c>
     </row>
     <row r="5">
@@ -1450,31 +1523,31 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="D5" t="n">
-        <v>10.5</v>
+        <v>2.75</v>
       </c>
       <c r="E5" t="n">
-        <v>1260</v>
+        <v>550</v>
       </c>
       <c r="F5" t="n">
-        <v>268.14</v>
+        <v>220.29</v>
       </c>
       <c r="G5" t="n">
-        <v>88.2</v>
+        <v>27.5</v>
       </c>
       <c r="H5" t="n">
-        <v>18.07</v>
+        <v>6.04</v>
       </c>
       <c r="I5" t="n">
-        <v>885.59</v>
+        <v>296.17</v>
       </c>
       <c r="J5" t="n">
         <v>34</v>
       </c>
       <c r="K5" t="n">
-        <v>26.05</v>
+        <v>8.710000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -1489,31 +1562,31 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="D6" t="n">
-        <v>11.25</v>
+        <v>2.9</v>
       </c>
       <c r="E6" t="n">
-        <v>900</v>
+        <v>348</v>
       </c>
       <c r="F6" t="n">
-        <v>194.1</v>
+        <v>133.83</v>
       </c>
       <c r="G6" t="n">
-        <v>45</v>
+        <v>13.92</v>
       </c>
       <c r="H6" t="n">
-        <v>13.22</v>
+        <v>4.01</v>
       </c>
       <c r="I6" t="n">
-        <v>647.6799999999999</v>
+        <v>196.25</v>
       </c>
       <c r="J6" t="n">
         <v>18</v>
       </c>
       <c r="K6" t="n">
-        <v>35.98</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="7">
@@ -1528,31 +1601,31 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="D7" t="n">
-        <v>11.25</v>
+        <v>2.9</v>
       </c>
       <c r="E7" t="n">
-        <v>4500</v>
+        <v>1740</v>
       </c>
       <c r="F7" t="n">
-        <v>970.5</v>
+        <v>669.15</v>
       </c>
       <c r="G7" t="n">
-        <v>225</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>66.09</v>
+        <v>20.03</v>
       </c>
       <c r="I7" t="n">
-        <v>3238.41</v>
+        <v>981.23</v>
       </c>
       <c r="J7" t="n">
         <v>45</v>
       </c>
       <c r="K7" t="n">
-        <v>71.95999999999999</v>
+        <v>21.81</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Re-date launch, validation and ops plans relative to the release gate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q1vimjhczAVgRxbbW9XqPG
</commit_message>
<xml_diff>
--- a/business/phd-atlas/ops/Business-Dashboard.xlsx
+++ b/business/phd-atlas/ops/Business-Dashboard.xlsx
@@ -225,12 +225,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Weekly actuals'!$A$2:$A$13</f>
+              <f>'Weekly actuals'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Weekly actuals'!$C$2:$C$13</f>
+              <f>'Weekly actuals'!$C$2:$C$17</f>
             </numRef>
           </val>
         </ser>
@@ -257,12 +257,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Weekly actuals'!$A$2:$A$13</f>
+              <f>'Weekly actuals'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Weekly actuals'!$D$2:$D$13</f>
+              <f>'Weekly actuals'!$D$2:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -322,7 +322,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>16</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="2880000"/>
@@ -655,7 +655,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>'Gates' turns green or red automatically against the Dec 15 decision rules.</t>
+          <t>'Gates' turns green or red automatically against the gate-review rules (6 weeks after launch).</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1060,69 +1060,153 @@
       <c r="Q13" s="5" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="4" t="n">
+        <v>46405</v>
+      </c>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
+      <c r="K14" s="5" t="n"/>
+      <c r="L14" s="5" t="n"/>
+      <c r="M14" s="5" t="n"/>
+      <c r="N14" s="5" t="n"/>
+      <c r="O14" s="5" t="n"/>
+      <c r="P14" s="5" t="n"/>
+      <c r="Q14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>46412</v>
+      </c>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
+      <c r="K15" s="5" t="n"/>
+      <c r="L15" s="5" t="n"/>
+      <c r="M15" s="5" t="n"/>
+      <c r="N15" s="5" t="n"/>
+      <c r="O15" s="5" t="n"/>
+      <c r="P15" s="5" t="n"/>
+      <c r="Q15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>46419</v>
+      </c>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
+      <c r="K16" s="5" t="n"/>
+      <c r="L16" s="5" t="n"/>
+      <c r="M16" s="5" t="n"/>
+      <c r="N16" s="5" t="n"/>
+      <c r="O16" s="5" t="n"/>
+      <c r="P16" s="5" t="n"/>
+      <c r="Q16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>46426</v>
+      </c>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="5" t="n"/>
+      <c r="K17" s="5" t="n"/>
+      <c r="L17" s="5" t="n"/>
+      <c r="M17" s="5" t="n"/>
+      <c r="N17" s="5" t="n"/>
+      <c r="O17" s="5" t="n"/>
+      <c r="P17" s="5" t="n"/>
+      <c r="Q17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B14" s="6">
-        <f>SUM(B2:B13)</f>
-        <v/>
-      </c>
-      <c r="C14" s="6">
-        <f>SUM(C2:C13)</f>
-        <v/>
-      </c>
-      <c r="D14" s="6">
-        <f>SUM(D2:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="6">
-        <f>SUM(E2:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="6">
-        <f>SUM(F2:F13)</f>
-        <v/>
-      </c>
-      <c r="G14" s="6">
-        <f>SUM(G2:G13)</f>
-        <v/>
-      </c>
-      <c r="H14" s="6">
-        <f>SUM(H2:H13)</f>
-        <v/>
-      </c>
-      <c r="I14" s="6">
-        <f>SUM(I2:I13)</f>
-        <v/>
-      </c>
-      <c r="J14" s="6">
-        <f>SUM(J2:J13)</f>
-        <v/>
-      </c>
-      <c r="K14" s="6">
-        <f>SUM(K2:K13)</f>
-        <v/>
-      </c>
-      <c r="L14" s="6">
-        <f>SUM(L2:L13)</f>
-        <v/>
-      </c>
-      <c r="M14" s="6">
-        <f>SUM(M2:M13)</f>
-        <v/>
-      </c>
-      <c r="N14" s="6">
-        <f>SUM(N2:N13)</f>
-        <v/>
-      </c>
-      <c r="O14" s="6">
-        <f>SUM(O2:O13)</f>
-        <v/>
-      </c>
-      <c r="P14" s="6">
-        <f>SUM(P2:P13)</f>
+      <c r="B18" s="6">
+        <f>SUM(B2:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="6">
+        <f>SUM(C2:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="6">
+        <f>SUM(D2:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="6">
+        <f>SUM(E2:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="6">
+        <f>SUM(F2:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="6">
+        <f>SUM(G2:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="6">
+        <f>SUM(H2:H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="6">
+        <f>SUM(I2:I17)</f>
+        <v/>
+      </c>
+      <c r="J18" s="6">
+        <f>SUM(J2:J17)</f>
+        <v/>
+      </c>
+      <c r="K18" s="6">
+        <f>SUM(K2:K17)</f>
+        <v/>
+      </c>
+      <c r="L18" s="6">
+        <f>SUM(L2:L17)</f>
+        <v/>
+      </c>
+      <c r="M18" s="6">
+        <f>SUM(M2:M17)</f>
+        <v/>
+      </c>
+      <c r="N18" s="6">
+        <f>SUM(N2:N17)</f>
+        <v/>
+      </c>
+      <c r="O18" s="6">
+        <f>SUM(O2:O17)</f>
+        <v/>
+      </c>
+      <c r="P18" s="6">
+        <f>SUM(P2:P17)</f>
         <v/>
       </c>
     </row>
@@ -1150,7 +1234,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Dec 15 gate</t>
+          <t>Gate review (launch + 6 weeks)</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
@@ -1181,7 +1265,7 @@
         </is>
       </c>
       <c r="C2">
-        <f>'Weekly actuals'!D14</f>
+        <f>'Weekly actuals'!D18</f>
         <v/>
       </c>
       <c r="D2">
@@ -1201,7 +1285,7 @@
         </is>
       </c>
       <c r="C3">
-        <f>'Weekly actuals'!E14</f>
+        <f>'Weekly actuals'!E18</f>
         <v/>
       </c>
       <c r="D3">
@@ -1221,11 +1305,11 @@
         </is>
       </c>
       <c r="C4" s="7">
-        <f>IF('Weekly actuals'!D14=0,0,'Weekly actuals'!F14/'Weekly actuals'!D14)</f>
+        <f>IF('Weekly actuals'!D18=0,0,'Weekly actuals'!F18/'Weekly actuals'!D18)</f>
         <v/>
       </c>
       <c r="D4">
-        <f>IF(AND('Weekly actuals'!D14&gt;0,C4&lt;=0.1),"PASS",IF('Weekly actuals'!D14=0,"no orders","FAIL"))</f>
+        <f>IF(AND('Weekly actuals'!D18&gt;0,C4&lt;=0.1),"PASS",IF('Weekly actuals'!D18=0,"no orders","FAIL"))</f>
         <v/>
       </c>
     </row>
@@ -1241,7 +1325,7 @@
         </is>
       </c>
       <c r="C5">
-        <f>'Weekly actuals'!L14</f>
+        <f>'Weekly actuals'!L18</f>
         <v/>
       </c>
       <c r="D5">
@@ -1261,7 +1345,7 @@
         </is>
       </c>
       <c r="C6">
-        <f>'Weekly actuals'!M14</f>
+        <f>'Weekly actuals'!M18</f>
         <v/>
       </c>
       <c r="D6">
@@ -1281,7 +1365,7 @@
         </is>
       </c>
       <c r="C7">
-        <f>'Weekly actuals'!C14</f>
+        <f>'Weekly actuals'!C18</f>
         <v/>
       </c>
       <c r="D7">
@@ -1292,7 +1376,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Decision (Dec 15)</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -2159,6 +2243,13 @@
         <v/>
       </c>
       <c r="E14" s="5" t="n"/>
+      <c r="G14" s="4" t="n">
+        <v>46405</v>
+      </c>
+      <c r="H14" s="9">
+        <f>SUMIF($D$2:$D$201,G14,$C$2:$C$201)/60</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n"/>
@@ -2169,6 +2260,13 @@
         <v/>
       </c>
       <c r="E15" s="5" t="n"/>
+      <c r="G15" s="4" t="n">
+        <v>46412</v>
+      </c>
+      <c r="H15" s="9">
+        <f>SUMIF($D$2:$D$201,G15,$C$2:$C$201)/60</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n"/>
@@ -2179,6 +2277,13 @@
         <v/>
       </c>
       <c r="E16" s="5" t="n"/>
+      <c r="G16" s="4" t="n">
+        <v>46419</v>
+      </c>
+      <c r="H16" s="9">
+        <f>SUMIF($D$2:$D$201,G16,$C$2:$C$201)/60</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n"/>
@@ -2189,6 +2294,13 @@
         <v/>
       </c>
       <c r="E17" s="5" t="n"/>
+      <c r="G17" s="4" t="n">
+        <v>46426</v>
+      </c>
+      <c r="H17" s="9">
+        <f>SUMIF($D$2:$D$201,G17,$C$2:$C$201)/60</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n"/>

</xml_diff>